<commit_message>
feat: updated MID code and appTests
</commit_message>
<xml_diff>
--- a/04 - MID/03 - Delete/01 - Demand/Data.xlsx
+++ b/04 - MID/03 - Delete/01 - Demand/Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mao8ct\Desktop\PyAutomateSAP\04 - MID\03 - Delete\01 - Demand\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{551DD812-C212-4683-AC8F-94566A389DE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EF2486C-F7C3-4CFB-8791-8B4ED13C46C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{841C4129-0CB3-4066-B34E-E8845E3509BE}"/>
   </bookViews>
@@ -439,44 +439,44 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
-        <v>685601397939</v>
+        <v>685601401883</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
-        <v>685601397938</v>
+        <v>685601401884</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
-        <v>685601397937</v>
+        <v>685601401885</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
-        <v>685601397936</v>
+        <v>685601401887</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
-        <v>685601397935</v>
+        <v>685601401890</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
-        <v>685601397934</v>
+        <v>685601401892</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
-        <v>685601397933</v>
+        <v>685601401894</v>
       </c>
       <c r="L8" s="3"/>
       <c r="M8" s="3"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
-        <v>685601397932</v>
+        <v>685601401895</v>
       </c>
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
@@ -485,7 +485,7 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
-        <v>685601397931</v>
+        <v>685601401896</v>
       </c>
       <c r="I10" s="3"/>
       <c r="J10" s="3"/>
@@ -494,7 +494,7 @@
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
-        <v>685601397930</v>
+        <v>685601401897</v>
       </c>
       <c r="I11" s="3"/>
       <c r="J11" s="3"/>
@@ -503,7 +503,7 @@
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
-        <v>685601397929</v>
+        <v>685601401898</v>
       </c>
       <c r="I12" s="3"/>
       <c r="J12" s="3"/>
@@ -511,61 +511,79 @@
       <c r="M12" s="3"/>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A13" s="2"/>
+      <c r="A13" s="2">
+        <v>685601401899</v>
+      </c>
       <c r="I13" s="3"/>
       <c r="J13" s="3"/>
       <c r="L13" s="3"/>
       <c r="M13" s="3"/>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A14" s="2"/>
+      <c r="A14" s="2">
+        <v>685601401900</v>
+      </c>
       <c r="I14" s="3"/>
       <c r="J14" s="3"/>
       <c r="L14" s="3"/>
       <c r="M14" s="3"/>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A15" s="2"/>
+      <c r="A15" s="2">
+        <v>685601401902</v>
+      </c>
       <c r="I15" s="3"/>
       <c r="J15" s="3"/>
       <c r="L15" s="3"/>
       <c r="M15" s="3"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A16" s="2"/>
+      <c r="A16" s="2">
+        <v>685601401903</v>
+      </c>
       <c r="I16" s="3"/>
       <c r="J16" s="3"/>
       <c r="L16" s="3"/>
       <c r="M16" s="3"/>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A17" s="2"/>
+      <c r="A17" s="2">
+        <v>685601401904</v>
+      </c>
       <c r="I17" s="3"/>
       <c r="J17" s="3"/>
       <c r="L17" s="3"/>
       <c r="M17" s="3"/>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A18" s="2"/>
+      <c r="A18" s="2">
+        <v>685601401905</v>
+      </c>
       <c r="I18" s="3"/>
       <c r="J18" s="3"/>
       <c r="L18" s="3"/>
       <c r="M18" s="3"/>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A19" s="2"/>
+      <c r="A19" s="2">
+        <v>685601401906</v>
+      </c>
       <c r="I19" s="3"/>
       <c r="J19" s="3"/>
       <c r="L19" s="3"/>
       <c r="M19" s="3"/>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A20" s="2"/>
+      <c r="A20" s="2">
+        <v>685601401907</v>
+      </c>
       <c r="L20" s="3"/>
       <c r="M20" s="3"/>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A21" s="2"/>
+      <c r="A21" s="2">
+        <v>685601401908</v>
+      </c>
       <c r="L21" s="3"/>
       <c r="M21" s="3"/>
     </row>

</xml_diff>

<commit_message>
used: delete demand bot
</commit_message>
<xml_diff>
--- a/04 - MID/03 - Delete/01 - Demand/Data.xlsx
+++ b/04 - MID/03 - Delete/01 - Demand/Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mao8ct\Desktop\PyAutomateSAP\04 - MID\03 - Delete\01 - Demand\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EF2486C-F7C3-4CFB-8791-8B4ED13C46C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C804234A-1015-4922-8513-910C46E91FFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{841C4129-0CB3-4066-B34E-E8845E3509BE}"/>
   </bookViews>
@@ -439,44 +439,44 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
-        <v>685601401883</v>
+        <v>685601403955</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
-        <v>685601401884</v>
+        <v>685601403956</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
-        <v>685601401885</v>
+        <v>685601403959</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
-        <v>685601401887</v>
+        <v>685601403960</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
-        <v>685601401890</v>
+        <v>685601403962</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
-        <v>685601401892</v>
+        <v>685601403963</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
-        <v>685601401894</v>
+        <v>685601403964</v>
       </c>
       <c r="L8" s="3"/>
       <c r="M8" s="3"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
-        <v>685601401895</v>
+        <v>685601403965</v>
       </c>
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
@@ -485,7 +485,7 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
-        <v>685601401896</v>
+        <v>685601403966</v>
       </c>
       <c r="I10" s="3"/>
       <c r="J10" s="3"/>
@@ -494,7 +494,7 @@
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
-        <v>685601401897</v>
+        <v>685601403966</v>
       </c>
       <c r="I11" s="3"/>
       <c r="J11" s="3"/>
@@ -503,7 +503,7 @@
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
-        <v>685601401898</v>
+        <v>685601403967</v>
       </c>
       <c r="I12" s="3"/>
       <c r="J12" s="3"/>
@@ -512,7 +512,7 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
-        <v>685601401899</v>
+        <v>685601403969</v>
       </c>
       <c r="I13" s="3"/>
       <c r="J13" s="3"/>
@@ -521,7 +521,7 @@
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
-        <v>685601401900</v>
+        <v>685601403973</v>
       </c>
       <c r="I14" s="3"/>
       <c r="J14" s="3"/>
@@ -529,61 +529,47 @@
       <c r="M14" s="3"/>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A15" s="2">
-        <v>685601401902</v>
-      </c>
+      <c r="A15" s="2"/>
       <c r="I15" s="3"/>
       <c r="J15" s="3"/>
       <c r="L15" s="3"/>
       <c r="M15" s="3"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A16" s="2">
-        <v>685601401903</v>
-      </c>
+      <c r="A16" s="2"/>
       <c r="I16" s="3"/>
       <c r="J16" s="3"/>
       <c r="L16" s="3"/>
       <c r="M16" s="3"/>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A17" s="2">
-        <v>685601401904</v>
-      </c>
+      <c r="A17" s="2"/>
       <c r="I17" s="3"/>
       <c r="J17" s="3"/>
       <c r="L17" s="3"/>
       <c r="M17" s="3"/>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A18" s="2">
-        <v>685601401905</v>
-      </c>
+      <c r="A18" s="2"/>
       <c r="I18" s="3"/>
       <c r="J18" s="3"/>
       <c r="L18" s="3"/>
       <c r="M18" s="3"/>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A19" s="2">
-        <v>685601401906</v>
-      </c>
+      <c r="A19" s="2"/>
       <c r="I19" s="3"/>
       <c r="J19" s="3"/>
       <c r="L19" s="3"/>
       <c r="M19" s="3"/>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A20" s="2">
-        <v>685601401907</v>
-      </c>
+      <c r="A20" s="2"/>
       <c r="L20" s="3"/>
       <c r="M20" s="3"/>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A21" s="2">
-        <v>685601401908</v>
-      </c>
+      <c r="A21" s="2"/>
       <c r="L21" s="3"/>
       <c r="M21" s="3"/>
     </row>

</xml_diff>